<commit_message>
Ajout de la feuille des résultats à l'import système (podiums, médailles automatiques)
</commit_message>
<xml_diff>
--- a/sample-imports/initialisation-systeme.xlsx
+++ b/sample-imports/initialisation-systeme.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Disciplines" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Epreuves" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Athletes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Resultats" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4652,7 +4653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4743,17 +4744,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Emma</t>
+          <t>Lucas</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Femme</t>
+          <t>Homme</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2009-02-02</t>
+          <t>2008-01-12</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -4763,7 +4764,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Aviron</t>
+          <t>Athlétisme</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -4791,7 +4792,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2010-03-03</t>
+          <t>2008-01-23</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -4801,7 +4802,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Badminton</t>
+          <t>Athlétisme</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -4829,7 +4830,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2011-04-04</t>
+          <t>2008-02-03</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -4839,7 +4840,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Basketball 3x3</t>
+          <t>Athlétisme</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -4857,17 +4858,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Omar</t>
+          <t>Fatima</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Homme</t>
+          <t>Femme</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2008-05-05</t>
+          <t>2008-02-14</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -4877,7 +4878,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Boxe</t>
+          <t>Athlétisme</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -4905,7 +4906,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2009-06-06</t>
+          <t>2008-02-25</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -4915,7 +4916,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Breaking</t>
+          <t>Athlétisme</t>
         </is>
       </c>
       <c r="G7" t="n">
@@ -4943,7 +4944,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2010-07-07</t>
+          <t>2008-03-07</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -4953,7 +4954,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Canoë-kayak</t>
+          <t>Natation</t>
         </is>
       </c>
       <c r="G8" t="n">
@@ -4971,17 +4972,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Lucia</t>
+          <t>Mateo</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Femme</t>
+          <t>Homme</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2011-08-08</t>
+          <t>2008-03-18</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -4991,7 +4992,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Cyclisme</t>
+          <t>Natation</t>
         </is>
       </c>
       <c r="G9" t="n">
@@ -5019,7 +5020,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2008-09-09</t>
+          <t>2008-03-29</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -5029,7 +5030,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Équitation</t>
+          <t>Natation</t>
         </is>
       </c>
       <c r="G10" t="n">
@@ -5057,7 +5058,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2009-10-10</t>
+          <t>2008-04-09</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -5067,7 +5068,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Escalade sportive</t>
+          <t>Natation</t>
         </is>
       </c>
       <c r="G11" t="n">
@@ -5085,17 +5086,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Ibrahim</t>
+          <t>Zineb</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Homme</t>
+          <t>Femme</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2010-11-11</t>
+          <t>2008-04-20</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -5105,7 +5106,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Escrime</t>
+          <t>Natation</t>
         </is>
       </c>
       <c r="G12" t="n">
@@ -5133,7 +5134,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2011-12-12</t>
+          <t>2008-05-01</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -5143,7 +5144,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Football</t>
+          <t>Natation</t>
         </is>
       </c>
       <c r="G13" t="n">
@@ -5171,7 +5172,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2008-01-13</t>
+          <t>2008-05-12</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -5181,7 +5182,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Golf</t>
+          <t>Judo</t>
         </is>
       </c>
       <c r="G14" t="n">
@@ -5199,17 +5200,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Ama</t>
+          <t>Kofi</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Femme</t>
+          <t>Homme</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2009-02-14</t>
+          <t>2008-05-23</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -5219,7 +5220,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Gymnastique artistique</t>
+          <t>Judo</t>
         </is>
       </c>
       <c r="G15" t="n">
@@ -5247,7 +5248,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2010-03-15</t>
+          <t>2008-06-03</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -5257,7 +5258,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Haltérophilie</t>
+          <t>Judo</t>
         </is>
       </c>
       <c r="G16" t="n">
@@ -5285,7 +5286,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2011-04-16</t>
+          <t>2008-06-14</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -5295,7 +5296,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Handball</t>
+          <t>Judo</t>
         </is>
       </c>
       <c r="G17" t="n">
@@ -5313,17 +5314,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Tariq</t>
+          <t>Layla</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Homme</t>
+          <t>Femme</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2008-05-17</t>
+          <t>2008-06-25</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -5333,7 +5334,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Hockey sur gazon</t>
+          <t>Judo</t>
         </is>
       </c>
       <c r="G18" t="n">
@@ -5361,7 +5362,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2009-06-18</t>
+          <t>2008-07-06</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -5399,7 +5400,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2010-07-19</t>
+          <t>2008-07-17</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -5409,7 +5410,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Karaté</t>
+          <t>Aviron</t>
         </is>
       </c>
       <c r="G20" t="n">
@@ -5437,7 +5438,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2011-08-20</t>
+          <t>2008-07-28</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -5447,7 +5448,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Lutte</t>
+          <t>Badminton</t>
         </is>
       </c>
       <c r="G21" t="n">
@@ -5475,7 +5476,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2008-09-21</t>
+          <t>2008-08-08</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -5485,7 +5486,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Natation</t>
+          <t>Basketball 3x3</t>
         </is>
       </c>
       <c r="G22" t="n">
@@ -5513,7 +5514,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2009-10-22</t>
+          <t>2008-08-19</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -5523,7 +5524,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Pentathlon moderne</t>
+          <t>Boxe</t>
         </is>
       </c>
       <c r="G23" t="n">
@@ -5551,7 +5552,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2010-11-23</t>
+          <t>2008-08-30</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -5561,7 +5562,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Rugby à sept</t>
+          <t>Breaking</t>
         </is>
       </c>
       <c r="G24" t="n">
@@ -5589,7 +5590,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2011-12-24</t>
+          <t>2008-09-10</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -5599,7 +5600,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Skateboard</t>
+          <t>Canoë-kayak</t>
         </is>
       </c>
       <c r="G25" t="n">
@@ -5627,7 +5628,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2008-01-25</t>
+          <t>2008-09-21</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -5637,7 +5638,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Taekwondo</t>
+          <t>Cyclisme</t>
         </is>
       </c>
       <c r="G26" t="n">
@@ -5665,7 +5666,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2009-02-26</t>
+          <t>2008-10-02</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -5675,7 +5676,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Tennis</t>
+          <t>Équitation</t>
         </is>
       </c>
       <c r="G27" t="n">
@@ -5703,7 +5704,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2010-03-27</t>
+          <t>2008-10-13</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -5713,7 +5714,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Tennis de table</t>
+          <t>Escalade sportive</t>
         </is>
       </c>
       <c r="G28" t="n">
@@ -5741,7 +5742,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2011-04-01</t>
+          <t>2008-10-24</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -5751,7 +5752,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Tir</t>
+          <t>Escrime</t>
         </is>
       </c>
       <c r="G29" t="n">
@@ -5779,7 +5780,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2008-05-02</t>
+          <t>2008-11-04</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -5789,7 +5790,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Tir à l'arc</t>
+          <t>Football</t>
         </is>
       </c>
       <c r="G30" t="n">
@@ -5817,7 +5818,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2009-06-03</t>
+          <t>2008-11-15</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -5827,7 +5828,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Triathlon</t>
+          <t>Golf</t>
         </is>
       </c>
       <c r="G31" t="n">
@@ -5855,7 +5856,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2010-07-04</t>
+          <t>2008-11-26</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -5865,7 +5866,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Voile</t>
+          <t>Gymnastique artistique</t>
         </is>
       </c>
       <c r="G32" t="n">
@@ -5893,7 +5894,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2011-08-05</t>
+          <t>2008-12-07</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -5903,7 +5904,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Volleyball de plage</t>
+          <t>Haltérophilie</t>
         </is>
       </c>
       <c r="G33" t="n">
@@ -5931,7 +5932,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2008-09-06</t>
+          <t>2008-12-18</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -5941,7 +5942,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Athlétisme</t>
+          <t>Handball</t>
         </is>
       </c>
       <c r="G34" t="n">
@@ -5969,7 +5970,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2009-10-07</t>
+          <t>2008-12-29</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -5979,7 +5980,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Aviron</t>
+          <t>Hockey sur gazon</t>
         </is>
       </c>
       <c r="G35" t="n">
@@ -6007,7 +6008,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2010-11-08</t>
+          <t>2009-01-09</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -6017,7 +6018,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Badminton</t>
+          <t>Karaté</t>
         </is>
       </c>
       <c r="G36" t="n">
@@ -6045,7 +6046,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2011-12-09</t>
+          <t>2009-01-20</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -6055,7 +6056,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Basketball 3x3</t>
+          <t>Lutte</t>
         </is>
       </c>
       <c r="G37" t="n">
@@ -6083,7 +6084,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>2008-01-10</t>
+          <t>2009-01-31</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -6093,7 +6094,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Boxe</t>
+          <t>Pentathlon moderne</t>
         </is>
       </c>
       <c r="G38" t="n">
@@ -6131,7 +6132,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Breaking</t>
+          <t>Rugby à sept</t>
         </is>
       </c>
       <c r="G39" t="n">
@@ -6159,7 +6160,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>2010-03-12</t>
+          <t>2009-02-22</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -6169,7 +6170,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Canoë-kayak</t>
+          <t>Skateboard</t>
         </is>
       </c>
       <c r="G40" t="n">
@@ -6197,7 +6198,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>2011-04-13</t>
+          <t>2009-03-05</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -6207,7 +6208,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Cyclisme</t>
+          <t>Taekwondo</t>
         </is>
       </c>
       <c r="G41" t="n">
@@ -6215,6 +6216,1793 @@
       </c>
       <c r="H41" t="n">
         <v>64</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Kowalski</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Amadou</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Homme</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>2009-03-16</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>GRN</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>170</v>
+      </c>
+      <c r="H42" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Silva</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Emma</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Femme</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>2009-03-27</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>NCA</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Tennis de table</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>171</v>
+      </c>
+      <c r="H43" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Andersson</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Kenji</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Homme</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>2009-04-07</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>VIN</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Tir</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>172</v>
+      </c>
+      <c r="H44" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Kim</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Sofia</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Femme</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>2009-04-18</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>AFG</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Tir à l'arc</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>173</v>
+      </c>
+      <c r="H45" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Hassan</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Omar</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Homme</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>2009-04-29</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>TPE</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Triathlon</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>174</v>
+      </c>
+      <c r="H46" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Ndiaye</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Olivia</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Femme</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>2009-05-10</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>JOR</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Voile</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>175</v>
+      </c>
+      <c r="H47" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Fernández</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Youssef</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Homme</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>2009-05-21</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LBN</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Volleyball de plage</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>176</v>
+      </c>
+      <c r="H48" t="n">
+        <v>71</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>epreuveLabel</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>discipline</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>athleteLastName</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>athleteFirstName</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>athleteBirthDate</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>100 m garçons</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Athlétisme</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Diallo</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Amadou</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2008-01-01</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>100 m garçons</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Athlétisme</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Martin</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Lucas</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2008-01-12</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>100 m garçons</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Athlétisme</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Tanaka</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Kenji</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2008-01-23</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>100 m filles</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Athlétisme</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-11-02</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>García</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Sofia</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2008-02-03</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>100 m filles</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Athlétisme</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-11-02</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Haddad</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Fatima</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2008-02-14</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>100 m filles</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Athlétisme</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-11-02</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Smith</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Olivia</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2008-02-25</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Saut en longueur garçons</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Athlétisme</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Diallo</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Amadou</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2008-01-01</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Saut en longueur garçons</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Athlétisme</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Martin</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Lucas</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2008-01-12</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Saut en longueur garçons</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Athlétisme</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Tanaka</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Kenji</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2008-01-23</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Saut en longueur filles</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Athlétisme</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-11-04</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>García</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Sofia</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2008-02-03</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Saut en longueur filles</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Athlétisme</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2026-11-04</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Haddad</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Fatima</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2008-02-14</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Saut en longueur filles</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Athlétisme</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2026-11-04</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Smith</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Olivia</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2008-02-25</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>50 m nage libre garçons</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Natation</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Ben Ali</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Youssef</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2008-03-07</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>50 m nage libre garçons</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Natation</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Rossi</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Mateo</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2008-03-18</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>50 m nage libre garçons</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Natation</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Nguyen</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Noah</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2008-03-29</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>50 m nage libre filles</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Natation</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2026-11-04</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Okafor</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Priya</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2008-04-09</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>50 m nage libre filles</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Natation</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2026-11-04</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Traoré</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Zineb</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2008-04-20</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>50 m nage libre filles</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Natation</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2026-11-04</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Dubois</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Chloé</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2008-05-01</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>100 m dos garçons</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Natation</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2026-11-05</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Ben Ali</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Youssef</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2008-03-07</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>100 m dos garçons</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Natation</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2026-11-05</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Rossi</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Mateo</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2008-03-18</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>100 m dos garçons</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Natation</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2026-11-05</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Nguyen</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Noah</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2008-03-29</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>100 m dos filles</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Natation</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2026-11-06</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Okafor</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Priya</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>2008-04-09</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>100 m dos filles</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Natation</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>2026-11-06</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Traoré</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Zineb</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2008-04-20</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>100 m dos filles</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Natation</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>2026-11-06</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Dubois</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Chloé</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2008-05-01</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>200 m 4 nages garçons</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Natation</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Ben Ali</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Youssef</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>2008-03-07</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>200 m 4 nages garçons</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Natation</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Rossi</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Mateo</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>2008-03-18</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>200 m 4 nages garçons</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Natation</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Nguyen</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Noah</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2008-03-29</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>200 m 4 nages filles</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Natation</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>2026-11-08</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Okafor</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Priya</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2008-04-09</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>200 m 4 nages filles</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Natation</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>2026-11-08</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Traoré</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Zineb</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2008-04-20</t>
+        </is>
+      </c>
+      <c r="G30" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>200 m 4 nages filles</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Natation</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>2026-11-08</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Dubois</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Chloé</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2008-05-01</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>-60 kg garçons</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Judo</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>2026-11-06</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Wang</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Chen</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>2008-05-12</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>-60 kg garçons</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Judo</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>2026-11-06</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Mensah</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Kofi</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2008-05-23</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>-60 kg garçons</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Judo</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>2026-11-06</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Petrov</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Andrei</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>2008-06-03</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>-60 kg filles</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Judo</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Kowalski</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Giulia</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>2008-06-14</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>-60 kg filles</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Judo</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Silva</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Layla</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>2008-06-25</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>-60 kg filles</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Judo</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Andersson</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Astrid</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>2008-07-06</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>-48 kg garçons</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Judo</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>2026-11-08</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Wang</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Chen</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>2008-05-12</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>-48 kg garçons</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Judo</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>2026-11-08</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Mensah</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Kofi</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>2008-05-23</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>-48 kg garçons</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Judo</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>2026-11-08</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Petrov</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Andrei</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>2008-06-03</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>-48 kg filles</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Judo</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Kowalski</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Giulia</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>2008-06-14</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>-48 kg filles</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Judo</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Silva</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Layla</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>2008-06-25</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>-48 kg filles</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Judo</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Andersson</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Astrid</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>2008-07-06</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>